<commit_message>
Files created through execution of Notebook 01 and 02
</commit_message>
<xml_diff>
--- a/makrooekonomische_indikatoren.xlsx
+++ b/makrooekonomische_indikatoren.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5d212592e769a8d3/Dokumente/_Studium/Bachelorarbeit/Analysis of macroeconomical indicators/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5d212592e769a8d3/Dokumente/_Studium/Bachelorarbeit/Practical Analysis/Explaining-Well-Being/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_BE6937031667C24FE3188837485DCE3A87C42D8A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90A4B482-C727-4391-8472-E464578CEDF4}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="11_BE6937031667C24FE3188837485DCE3A87C42D8A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{895D2E94-6C18-4B4B-8314-3EA4064EC911}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -355,7 +355,7 @@
     <t>Erwerbsquote (Männer): Anteil der Männer, die dem Arbeitsmarkt zur Verfügung stehen.</t>
   </si>
   <si>
-    <t>Beibehaltene Indikatoren der WISE Databse</t>
+    <t>Makroökonomische Indikatoren der WISE Databse</t>
   </si>
 </sst>
 </file>

</xml_diff>